<commit_message>
fix: remove doc_ids column from queries_type_3_4 Excel, match exact 5-column format of 1256 file
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/evaluation/queries_type_3_4_before_pooling.xlsx
+++ b/data/evaluation/queries_type_3_4_before_pooling.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,11 +442,6 @@
           <t>notes</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>doc_ids</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -454,8 +449,10 @@
           <t>Deep_Query_1</t>
         </is>
       </c>
-      <c r="B2" t="n">
-        <v>3</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -468,11 +465,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>["NK-ntNa6xcjdwGRXzxV6wpxfd", "NK-cfWFCgJ7etMfnZSJx4xSsb", "NK-GFtNiBqrmJG8ofBNQt97hF", "NK-Wv2e4rkvjjKptipYph5nv7", "NK-SCWNRatvQgpQFUnd8zS4A7", "NK-irZCKsygfBbdat8u2JB7ui", "NK-cxdpQ8HhWX9XXLq9zVonUB", "NK-UN2ZMUxjk6ZYNP5bqyUUxe", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy"]</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -480,8 +472,10 @@
           <t>Deep_Query_2</t>
         </is>
       </c>
-      <c r="B3" t="n">
-        <v>3</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -494,11 +488,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>["NK-MYHWYA7zLoQoGrPfVPUcYt", "NK-MVtCt6RAzxf245XiueFWJp", "NK-EQ3dGe5XJhvdMYtQfvKVsP", "kprusi-6bf4f6bf84f9b42a737a9bdf27e84bae9f396585", "NK-Xv8CnM8sgddxx7QenotGtb"]</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -506,8 +495,10 @@
           <t>Deep_Query_3</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>3</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -520,11 +511,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>["NK-fjaabCsg83J67wd2T3LXoP", "NK-EL5cFqL5pRrFRBSUjny38g", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy"]</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -532,8 +518,10 @@
           <t>Deep_Query_4</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>3</v>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -546,11 +534,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>["NK-Wv2e4rkvjjKptipYph5nv7", "NK-ZHdpKQLko7n8ZSsM2RS37N", "NK-PpgkyRStFVvftErWkkLxtW"]</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -558,8 +541,10 @@
           <t>Deep_Query_5</t>
         </is>
       </c>
-      <c r="B6" t="n">
-        <v>3</v>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -572,11 +557,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>["NK-EL5cFqL5pRrFRBSUjny38g", "NK-B95TF42hNDRBtmaRrW4wwp", "Q112041861", "NK-eXzFarXNX73XPhYRp9xM33"]</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -584,8 +564,10 @@
           <t>Deep_Query_6</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>4</v>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -598,11 +580,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>["NK-EL5cFqL5pRrFRBSUjny38g", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy", "NK-B95TF42hNDRBtmaRrW4wwp", "NK-fjaabCsg83J67wd2T3LXoP"]</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -610,8 +587,10 @@
           <t>Deep_Query_7</t>
         </is>
       </c>
-      <c r="B8" t="n">
-        <v>4</v>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -624,11 +603,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>["NK-MYHWYA7zLoQoGrPfVPUcYt", "NK-MVtCt6RAzxf245XiueFWJp", "NK-EQ3dGe5XJhvdMYtQfvKVsP", "kprusi-6bf4f6bf84f9b42a737a9bdf27e84bae9f396585", "NK-Xv8CnM8sgddxx7QenotGtb"]</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -636,8 +610,10 @@
           <t>Deep_Query_8</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>4</v>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -650,11 +626,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>["NK-EL5cFqL5pRrFRBSUjny38g", "NK-B95TF42hNDRBtmaRrW4wwp", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy", "NK-eXzFarXNX73XPhYRp9xM33", "Q112041861", "NK-fjaabCsg83J67wd2T3LXoP"]</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -662,8 +633,10 @@
           <t>Deep_Query_9</t>
         </is>
       </c>
-      <c r="B10" t="n">
-        <v>4</v>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -676,11 +649,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>["NK-fjaabCsg83J67wd2T3LXoP", "NK-EL5cFqL5pRrFRBSUjny38g", "NK-FoHPKahRH6oYTxbT7Tycjk", "NK-AJdA3Gt5CuYSxKVuUAfQfy"]</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -688,8 +656,10 @@
           <t>Deep_Query_10</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>4</v>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -702,11 +672,6 @@
           <t>SHADOW FLEET / DPRK CYBER / UAE SHELL MGMT</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>["NK-EL5cFqL5pRrFRBSUjny38g", "Q112041861", "NK-eXzFarXNX73XPhYRp9xM33"]</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -714,8 +679,10 @@
           <t>Deep_Query_11</t>
         </is>
       </c>
-      <c r="B12" t="n">
-        <v>3</v>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -728,11 +695,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>["Q36597284", "NK-Z9oNBzxf4NzcB6GKXwgPUL", "Q20850503", "NK-SGoKLj97jDeyJGnSyRhJJN", "NK-h2aV4Qyf26ZsX33pRzHRDc"]</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -740,8 +702,10 @@
           <t>Deep_Query_12</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>3</v>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -754,11 +718,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>["NK-cuVFsKgk3rPqzM4pWTexzc", "NK-N7dfJjNtqB9hibmDaoviPf", "NK-3MPTNLvV5pezgcPmtqapAM"]</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -766,8 +725,10 @@
           <t>Deep_Query_13</t>
         </is>
       </c>
-      <c r="B14" t="n">
-        <v>3</v>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -780,11 +741,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>["Q120852793", "Q36597284", "Q20850503"]</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -792,8 +748,10 @@
           <t>Deep_Query_14</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>3</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -806,11 +764,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>["NK-mFuJH7pUGnr7fegsQYbRWp", "NK-TsnsTYDD5QeZ9gDbFB2WbU", "NK-N7dfJjNtqB9hibmDaoviPf"]</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -818,8 +771,10 @@
           <t>Deep_Query_15</t>
         </is>
       </c>
-      <c r="B16" t="n">
-        <v>3</v>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -832,11 +787,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>["NK-SGoKLj97jDeyJGnSyRhJJN", "Q107586452", "Q36597284"]</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -844,8 +794,10 @@
           <t>Deep_Query_16</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>4</v>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -858,11 +810,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>["Q36597284", "NK-Z9oNBzxf4NzcB6GKXwgPUL", "Q20850503", "NK-SGoKLj97jDeyJGnSyRhJJN", "NK-h2aV4Qyf26ZsX33pRzHRDc", "Q120853746", "Q107586452"]</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -870,8 +817,10 @@
           <t>Deep_Query_17</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>4</v>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -884,11 +833,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>["Q120852793", "NK-N7dfJjNtqB9hibmDaoviPf", "NK-TsnsTYDD5QeZ9gDbFB2WbU", "NK-3MPTNLvV5pezgcPmtqapAM", "NK-mFuJH7pUGnr7fegsQYbRWp", "NK-8H4ADaELozj4fx4NYAYZjF", "NK-n8gyfuPWedBXSbpTnLarj8", "NK-YHHfaWGJ4rhJczQmJrZVfC", "NK-Za9Z4Nz5aGAWsd3B8H4VrT"]</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -896,8 +840,10 @@
           <t>Deep_Query_18</t>
         </is>
       </c>
-      <c r="B19" t="n">
-        <v>4</v>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -910,11 +856,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>["Q20850503", "Q36597284", "NK-Z9oNBzxf4NzcB6GKXwgPUL", "Q120852793"]</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -922,8 +863,10 @@
           <t>Deep_Query_19</t>
         </is>
       </c>
-      <c r="B20" t="n">
-        <v>4</v>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -936,11 +879,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>["NK-SGoKLj97jDeyJGnSyRhJJN", "Q107586452", "Q36597284", "Q20850503"]</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -948,8 +886,10 @@
           <t>Deep_Query_20</t>
         </is>
       </c>
-      <c r="B21" t="n">
-        <v>4</v>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -962,11 +902,6 @@
           <t>WAGNER PMC / GAZPROM ENERGY</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>["Q36597284", "Q120853746", "Q120852793", "Q20850503"]</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -974,8 +909,10 @@
           <t>Deep_Query_21</t>
         </is>
       </c>
-      <c r="B22" t="n">
-        <v>3</v>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -988,11 +925,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>["NK-mZimbPviBCZ8d7BeGeK5nQ", "NK-nxAfGhdZUyo6cQJ6vVibxz", "NK-Gn2TD79skZ3tSjuXvPmMfZ", "NK-6mWPPVmJzBchaEjgzqcZeB", "NK-kNULoiM7XfTYeWLtTZ4UHg", "NK-jLcvcAFxBd2aYNeqUvit3a", "NK-hQEF3vmPJKUQshxZRMEEgo", "NK-9iiiphJsGDHoyN8WZuof3Q", "NK-MkLoWstKvmwk5LKkKiWepk"]</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1000,8 +932,10 @@
           <t>Deep_Query_22</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>4</v>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1014,11 +948,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>["NK-kNULoiM7XfTYeWLtTZ4UHg", "NK-jLcvcAFxBd2aYNeqUvit3a", "NK-hQEF3vmPJKUQshxZRMEEgo", "NK-9iiiphJsGDHoyN8WZuof3Q"]</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1026,8 +955,10 @@
           <t>Deep_Query_23</t>
         </is>
       </c>
-      <c r="B24" t="n">
-        <v>4</v>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1040,11 +971,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>["NK-mZimbPviBCZ8d7BeGeK5nQ", "NK-nxAfGhdZUyo6cQJ6vVibxz", "NK-6mWPPVmJzBchaEjgzqcZeB", "NK-MkLoWstKvmwk5LKkKiWepk", "NK-Gn2TD79skZ3tSjuXvPmMfZ"]</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1052,8 +978,10 @@
           <t>Deep_Query_24</t>
         </is>
       </c>
-      <c r="B25" t="n">
-        <v>3</v>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1066,11 +994,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>["NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-f8wa3QmkpZDMtjiA6AkMns", "NK-AmRGwyzifJDB2PHBJTGyyM", "NK-jF6xZDZzsiGDtJtGcBqoLi", "NK-f24scmxDu6J7gRYcS6nbKt"]</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1078,8 +1001,10 @@
           <t>Deep_Query_25</t>
         </is>
       </c>
-      <c r="B26" t="n">
-        <v>3</v>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1092,11 +1017,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>["Q461631", "NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-jF6xZDZzsiGDtJtGcBqoLi"]</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1104,8 +1024,10 @@
           <t>Deep_Query_26</t>
         </is>
       </c>
-      <c r="B27" t="n">
-        <v>4</v>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1118,11 +1040,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>["NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-f8wa3QmkpZDMtjiA6AkMns", "NK-AmRGwyzifJDB2PHBJTGyyM", "NK-jF6xZDZzsiGDtJtGcBqoLi", "NK-f24scmxDu6J7gRYcS6nbKt", "Q461631", "NK-eih3utdAN5JxttKvdA2C7y"]</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1130,8 +1047,10 @@
           <t>Deep_Query_27</t>
         </is>
       </c>
-      <c r="B28" t="n">
-        <v>4</v>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1144,11 +1063,6 @@
           <t>DUAL-USE TECHNOLOGY / IRANIAN DRONES</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>["NK-jF6xZDZzsiGDtJtGcBqoLi", "NK-Nz46UHrXiSCEWLkEQTdoPb", "NK-f8wa3QmkpZDMtjiA6AkMns", "NK-AmRGwyzifJDB2PHBJTGyyM", "NK-f24scmxDu6J7gRYcS6nbKt", "NK-eih3utdAN5JxttKvdA2C7y"]</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1156,8 +1070,10 @@
           <t>Deep_Query_28</t>
         </is>
       </c>
-      <c r="B29" t="n">
-        <v>3</v>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1170,11 +1086,6 @@
           <t>Other_misc_queries</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>["NK-Xv8CnM8sgddxx7QenotGtb", "fbi-lazarus-2876490857c62ddcf8bf089eebd691ed739074dc", "fbi-lazarus-16600ec2ce87bbe1d621bc8a49126cdbd941ae80", "fbi-lazarus-3d52db0cd5be811f997a3c478bc7548690ed85a2", "fbi-lazarus-190b60b8a64fdc41c4468b99f47750d611523ae8", "fbi-lazarus-361c34aeea7771f0c4ae91d97f8769b07d6931c3", "fbi-lazarus-240bb5407be646f7f768d35f0ceb547945d96c8d", "fbi-lazarus-4f05d698ddad088da2e2ce2bf93b6073c93241c5", "fbi-lazarus-55e66b1975218a062a36f86b3d2483c82c265742", "fbi-lazarus-204f6c38bd61b2bda3c864a7eccbf7b0a14f8e57", "fbi-lazarus-19b06e8cd602f407780c2abf2ae1099e70adcdcf"]</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1182,8 +1093,10 @@
           <t>Deep_Query_29</t>
         </is>
       </c>
-      <c r="B30" t="n">
-        <v>3</v>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1196,11 +1109,6 @@
           <t>Other_misc_queries</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>["NK-YZDkBfVz9siwsep35GFbiF", "NK-5W6hj6czEXYyFJwTQ7g9ux", "NK-o8VasJ9pUxsVdhwQeB2b9P"]</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1208,8 +1116,10 @@
           <t>Deep_Query_30</t>
         </is>
       </c>
-      <c r="B31" t="n">
-        <v>3</v>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1222,11 +1132,6 @@
           <t>Other_misc_queries</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>["NK-BWSfTq3iX7YzFrwPyiszKh", "NK-nCCRCEZeb4t4Rz8QxUji3C", "NK-4fa3SNWJz2XnjbgGNGKmM7"]</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1234,8 +1139,10 @@
           <t>Deep_Query_31</t>
         </is>
       </c>
-      <c r="B32" t="n">
-        <v>3</v>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1248,11 +1155,6 @@
           <t>Other_misc_queries</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>["NK-3JmgoFcWsskLYxazEtcLe2", "NK-YofLoM3xwC3KVyAAVdBukG", "NK-bLCxB6FeXgQDisvnGdfMFR", "NK-MuEMnWHdG4nvov8oSJQMQS", "NK-itTPWRQCo37L7oLLw829aA", "NK-7Zp5k9c3BAT2yRFjpewJjx", "NK-FhbRxgHe8GGoGc3Lj4owXm"]</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1260,8 +1162,10 @@
           <t>Deep_Query_32</t>
         </is>
       </c>
-      <c r="B33" t="n">
-        <v>3</v>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1272,11 +1176,6 @@
       <c r="E33" t="inlineStr">
         <is>
           <t>Other_misc_queries</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>["NK-DTsY5n5CASmFd4Kd8FE7Ho", "NK-6wX7MJ9Aza8DYDu2EQ4Ztm", "NK-G4QXP35QijVQdaXtXpLhds"]</t>
         </is>
       </c>
     </row>

</xml_diff>